<commit_message>
Highlight missing Excel cells in yellow
</commit_message>
<xml_diff>
--- a/輸出檔/0414官網上架匯入收音機的檔案/0414新品-推薦(待填寫).xlsx
+++ b/輸出檔/0414官網上架匯入收音機的檔案/0414新品-推薦(待填寫).xlsx
@@ -29,7 +29,7 @@
       <b val="1"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill/>
     </fill>
@@ -39,6 +39,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00D9EAF7"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFF2CC"/>
       </patternFill>
     </fill>
   </fills>
@@ -54,11 +59,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -455,8 +461,8 @@
           <t>P33034</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr"/>
-      <c r="C2" t="inlineStr"/>
+      <c r="B2" s="2" t="inlineStr"/>
+      <c r="C2" s="2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -464,8 +470,8 @@
           <t>P33061</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr"/>
-      <c r="C3" t="inlineStr"/>
+      <c r="B3" s="2" t="inlineStr"/>
+      <c r="C3" s="2" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -473,8 +479,8 @@
           <t>P33103</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr"/>
-      <c r="C4" t="inlineStr"/>
+      <c r="B4" s="2" t="inlineStr"/>
+      <c r="C4" s="2" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -482,8 +488,8 @@
           <t>P33104</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr"/>
-      <c r="C5" t="inlineStr"/>
+      <c r="B5" s="2" t="inlineStr"/>
+      <c r="C5" s="2" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -491,8 +497,8 @@
           <t>P33115</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr"/>
-      <c r="C6" t="inlineStr"/>
+      <c r="B6" s="2" t="inlineStr"/>
+      <c r="C6" s="2" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -500,8 +506,8 @@
           <t>P33232</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr"/>
-      <c r="C7" t="inlineStr"/>
+      <c r="B7" s="2" t="inlineStr"/>
+      <c r="C7" s="2" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -509,8 +515,8 @@
           <t>P33282</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr"/>
-      <c r="C8" t="inlineStr"/>
+      <c r="B8" s="2" t="inlineStr"/>
+      <c r="C8" s="2" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -518,8 +524,8 @@
           <t>P33296</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr"/>
-      <c r="C9" t="inlineStr"/>
+      <c r="B9" s="2" t="inlineStr"/>
+      <c r="C9" s="2" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -527,8 +533,8 @@
           <t>P33089</t>
         </is>
       </c>
-      <c r="B10" t="inlineStr"/>
-      <c r="C10" t="inlineStr"/>
+      <c r="B10" s="2" t="inlineStr"/>
+      <c r="C10" s="2" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -536,8 +542,8 @@
           <t>P32990</t>
         </is>
       </c>
-      <c r="B11" t="inlineStr"/>
-      <c r="C11" t="inlineStr"/>
+      <c r="B11" s="2" t="inlineStr"/>
+      <c r="C11" s="2" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>